<commit_message>
prodcution api and new api for inventory hold
</commit_message>
<xml_diff>
--- a/PixelTracks_API_Documentation.xlsx
+++ b/PixelTracks_API_Documentation.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1398" uniqueCount="290">
   <si>
     <t>Pixel Tracks Backend — API Documentation</t>
   </si>
@@ -266,6 +266,120 @@
     <t>Delete an order by ID</t>
   </si>
   <si>
+    <t>— Products —</t>
+  </si>
+  <si>
+    <t>Products</t>
+  </si>
+  <si>
+    <t>/api/products</t>
+  </si>
+  <si>
+    <t>http://localhost:8000/api/products</t>
+  </si>
+  <si>
+    <t>Get all products (supplier configurations)</t>
+  </si>
+  <si>
+    <t>/api/products/:id</t>
+  </si>
+  <si>
+    <t>http://localhost:8000/api/products/:id</t>
+  </si>
+  <si>
+    <t>Get a single product</t>
+  </si>
+  <si>
+    <t>Create a new product configuration</t>
+  </si>
+  <si>
+    <t>400 Missing fields | 500 Database error</t>
+  </si>
+  <si>
+    <t>Update a product configuration</t>
+  </si>
+  <si>
+    <t>Delete a product</t>
+  </si>
+  <si>
+    <t>— Inventory —</t>
+  </si>
+  <si>
+    <t>Inventory</t>
+  </si>
+  <si>
+    <t>/api/inventory</t>
+  </si>
+  <si>
+    <t>http://localhost:8000/api/inventory</t>
+  </si>
+  <si>
+    <t>Get all inventory items, calculated available quantities, and holds</t>
+  </si>
+  <si>
+    <t>/api/inventory/:id</t>
+  </si>
+  <si>
+    <t>http://localhost:8000/api/inventory/:id</t>
+  </si>
+  <si>
+    <t>Get single inventory item</t>
+  </si>
+  <si>
+    <t>Create new inventory record</t>
+  </si>
+  <si>
+    <t>Update an inventory record</t>
+  </si>
+  <si>
+    <t>Delete inventory record</t>
+  </si>
+  <si>
+    <t>— Production —</t>
+  </si>
+  <si>
+    <t>Production</t>
+  </si>
+  <si>
+    <t>/api/production</t>
+  </si>
+  <si>
+    <t>http://localhost:8000/api/production</t>
+  </si>
+  <si>
+    <t>Get all production records with nested inventory item details</t>
+  </si>
+  <si>
+    <t>Create a production request manually</t>
+  </si>
+  <si>
+    <t>/api/production/request</t>
+  </si>
+  <si>
+    <t>http://localhost:8000/api/production/request</t>
+  </si>
+  <si>
+    <t>Auto-create production requests for an order (Step 1 &amp; Step 2)</t>
+  </si>
+  <si>
+    <t>/api/production/:id/status</t>
+  </si>
+  <si>
+    <t>http://localhost:8000/api/production/:id/status</t>
+  </si>
+  <si>
+    <t>Update production status and manage inventory holds/completions</t>
+  </si>
+  <si>
+    <t>/api/production/:id</t>
+  </si>
+  <si>
+    <t>http://localhost:8000/api/production/:id</t>
+  </si>
+  <si>
+    <t>Delete a production record and release holds</t>
+  </si>
+  <si>
     <t>Pixel Tracks Backend — Parameters Detail</t>
   </si>
   <si>
@@ -603,6 +717,171 @@
   </si>
   <si>
     <t>{ message: "Order deleted successfully" }</t>
+  </si>
+  <si>
+    <t>{ data: [...products] }</t>
+  </si>
+  <si>
+    <t>Product ID</t>
+  </si>
+  <si>
+    <t>{ data: { ...product } }</t>
+  </si>
+  <si>
+    <t>manufacturer</t>
+  </si>
+  <si>
+    <t>Supplier name</t>
+  </si>
+  <si>
+    <t>Color name</t>
+  </si>
+  <si>
+    <t>color_code</t>
+  </si>
+  <si>
+    <t>Color code</t>
+  </si>
+  <si>
+    <t>full_roll_length</t>
+  </si>
+  <si>
+    <t>Length of full roll</t>
+  </si>
+  <si>
+    <t>slits_per_roll</t>
+  </si>
+  <si>
+    <t>Number of slits</t>
+  </si>
+  <si>
+    <t>slitted_roll_length</t>
+  </si>
+  <si>
+    <t>Length of slitted roll</t>
+  </si>
+  <si>
+    <t>{ message: "Product created", data: { ...product } }</t>
+  </si>
+  <si>
+    <t>{ message: "Product updated", data: { ...product } }</t>
+  </si>
+  <si>
+    <t>{ message: "Product deleted" }</t>
+  </si>
+  <si>
+    <t>{ data: [...inventoryItems] }</t>
+  </si>
+  <si>
+    <t>Inventory ID</t>
+  </si>
+  <si>
+    <t>{ data: { ...inventoryItem } }</t>
+  </si>
+  <si>
+    <t>supplier</t>
+  </si>
+  <si>
+    <t>color_name</t>
+  </si>
+  <si>
+    <t>inventory_type</t>
+  </si>
+  <si>
+    <t>Full Roll | Slitted | Ready Channel</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>For rolls</t>
+  </si>
+  <si>
+    <t>size</t>
+  </si>
+  <si>
+    <t>pieces</t>
+  </si>
+  <si>
+    <t>For ready channels</t>
+  </si>
+  <si>
+    <t>length</t>
+  </si>
+  <si>
+    <t>{ message: "Inventory added", data: { ...item } }</t>
+  </si>
+  <si>
+    <t>{ message: "Inventory updated", data: { ...item } }</t>
+  </si>
+  <si>
+    <t>{ message: "Inventory deleted" }</t>
+  </si>
+  <si>
+    <t>{ data: [...productionList] }</t>
+  </si>
+  <si>
+    <t>production_type</t>
+  </si>
+  <si>
+    <t>General Inventory | Specific Order</t>
+  </si>
+  <si>
+    <t>raw_material_id</t>
+  </si>
+  <si>
+    <t>Inventory ID to hold</t>
+  </si>
+  <si>
+    <t>target_state</t>
+  </si>
+  <si>
+    <t>Ready Channel | Slitted</t>
+  </si>
+  <si>
+    <t>qty</t>
+  </si>
+  <si>
+    <t>Amount to hold</t>
+  </si>
+  <si>
+    <t>waste_qty</t>
+  </si>
+  <si>
+    <t>Estimated waste</t>
+  </si>
+  <si>
+    <t>{ message: "Production request created", data: { ...prod } }</t>
+  </si>
+  <si>
+    <t>order_id</t>
+  </si>
+  <si>
+    <t>Order ID</t>
+  </si>
+  <si>
+    <t>plan</t>
+  </si>
+  <si>
+    <t>Object</t>
+  </si>
+  <si>
+    <t>Satisfaction plan from calculateInventorySatisfaction</t>
+  </si>
+  <si>
+    <t>{ message: "Production requests created successfully" }</t>
+  </si>
+  <si>
+    <t>Production ID</t>
+  </si>
+  <si>
+    <t>In Progress | Completed | Cancelled</t>
+  </si>
+  <si>
+    <t>{ message: "Status updated to Completed" }</t>
+  </si>
+  <si>
+    <t>{ message: "Deleted successfully" }</t>
   </si>
 </sst>
 </file>
@@ -1208,7 +1487,7 @@
   <sheetPr>
     <tabColor rgb="FF1E3A5F"/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1814,14 +2093,443 @@
         <v>47</v>
       </c>
     </row>
+    <row r="28" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
+    </row>
+    <row r="29" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B29" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D29" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="E29" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="F29" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="G29" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H29" s="16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B30" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="G30" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H30" s="11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="E31" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="F31" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="G31" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="H31" s="16" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B32" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="G32" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H32" s="11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="F33" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="G33" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H33" s="16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
+    </row>
+    <row r="35" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B35" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G35" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H35" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="B36" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="E36" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="F36" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="G36" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H36" s="16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G37" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="H37" s="11" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="B38" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="E38" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="F38" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="G38" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H38" s="16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B39" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="F39" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="G39" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H39" s="11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4"/>
+      <c r="H40" s="4"/>
+    </row>
+    <row r="41" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="B41" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C41" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="D41" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="E41" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="F41" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="G41" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H41" s="16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D42" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G42" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="H42" s="11" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="D43" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="E43" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="F43" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="G43" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="H43" s="16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B44" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="E44" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="G44" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H44" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="B45" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="C45" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="D45" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="E45" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="F45" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="G45" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H45" s="16" t="s">
+        <v>47</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="9">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A40:H40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1833,7 +2541,7 @@
   <sheetPr>
     <tabColor rgb="FF2E86AB"/>
   </sheetPr>
-  <dimension ref="A1:H114"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1847,7 +2555,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>84</v>
+        <v>122</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1884,13 +2592,13 @@
         <v>7</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>85</v>
+        <v>123</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>6</v>
@@ -1922,62 +2630,62 @@
         <v>16</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>88</v>
+        <v>126</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G6" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>90</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>92</v>
+        <v>130</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>93</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F8" s="26" t="s">
-        <v>96</v>
+        <v>134</v>
       </c>
       <c r="G8" s="26"/>
       <c r="H8" s="26"/>
@@ -1996,62 +2704,62 @@
         <v>16</v>
       </c>
       <c r="E10" s="27" t="s">
-        <v>88</v>
+        <v>126</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H10" s="15" t="s">
-        <v>97</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>92</v>
+        <v>130</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H11" s="15" t="s">
-        <v>98</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D12" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E12" s="25" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F12" s="26" t="s">
-        <v>99</v>
+        <v>137</v>
       </c>
       <c r="G12" s="26"/>
       <c r="H12" s="26"/>
@@ -2082,62 +2790,62 @@
         <v>16</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>100</v>
+        <v>138</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>101</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C16" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>102</v>
+        <v>140</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>103</v>
+        <v>141</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B17" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C17" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D17" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E17" s="25" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F17" s="26" t="s">
-        <v>104</v>
+        <v>142</v>
       </c>
       <c r="G17" s="26"/>
       <c r="H17" s="26"/>
@@ -2156,36 +2864,36 @@
         <v>33</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>105</v>
+        <v>143</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>105</v>
+        <v>143</v>
       </c>
       <c r="G19" s="30" t="s">
         <v>33</v>
       </c>
       <c r="H19" s="15" t="s">
-        <v>106</v>
+        <v>144</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B20" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C20" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E20" s="25" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F20" s="26" t="s">
-        <v>107</v>
+        <v>145</v>
       </c>
       <c r="G20" s="26"/>
       <c r="H20" s="26"/>
@@ -2204,140 +2912,140 @@
         <v>16</v>
       </c>
       <c r="E22" s="22" t="s">
-        <v>100</v>
+        <v>138</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G22" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>108</v>
+        <v>146</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C23" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>102</v>
+        <v>140</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G23" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>109</v>
+        <v>147</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C24" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E24" s="22" t="s">
-        <v>110</v>
+        <v>148</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G24" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>111</v>
+        <v>149</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C25" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>112</v>
+        <v>150</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G25" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>114</v>
+        <v>152</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C26" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E26" s="22" t="s">
-        <v>115</v>
+        <v>153</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G26" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>116</v>
+        <v>154</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B27" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C27" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D27" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E27" s="25" t="s">
-        <v>117</v>
+        <v>155</v>
       </c>
       <c r="F27" s="26" t="s">
-        <v>118</v>
+        <v>156</v>
       </c>
       <c r="G27" s="26"/>
       <c r="H27" s="26"/>
@@ -2356,166 +3064,166 @@
         <v>42</v>
       </c>
       <c r="E29" s="27" t="s">
-        <v>119</v>
+        <v>157</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>120</v>
+        <v>158</v>
       </c>
       <c r="G29" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H29" s="15" t="s">
-        <v>121</v>
+        <v>159</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C30" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E30" s="27" t="s">
-        <v>100</v>
+        <v>138</v>
       </c>
       <c r="F30" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G30" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H30" s="15" t="s">
-        <v>122</v>
+        <v>160</v>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C31" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E31" s="27" t="s">
-        <v>102</v>
+        <v>140</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G31" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H31" s="15" t="s">
-        <v>123</v>
+        <v>161</v>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C32" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E32" s="27" t="s">
-        <v>110</v>
+        <v>148</v>
       </c>
       <c r="F32" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G32" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H32" s="15" t="s">
-        <v>124</v>
+        <v>162</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C33" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E33" s="27" t="s">
-        <v>112</v>
+        <v>150</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G33" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H33" s="15" t="s">
-        <v>125</v>
+        <v>163</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C34" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E34" s="27" t="s">
-        <v>115</v>
+        <v>153</v>
       </c>
       <c r="F34" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G34" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H34" s="15" t="s">
-        <v>126</v>
+        <v>164</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B35" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C35" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D35" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E35" s="25" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F35" s="26" t="s">
-        <v>127</v>
+        <v>165</v>
       </c>
       <c r="G35" s="26"/>
       <c r="H35" s="26"/>
@@ -2534,36 +3242,36 @@
         <v>46</v>
       </c>
       <c r="E37" s="22" t="s">
-        <v>119</v>
+        <v>157</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>120</v>
+        <v>158</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H37" s="9" t="s">
-        <v>128</v>
+        <v>166</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B38" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C38" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D38" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E38" s="25" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F38" s="26" t="s">
-        <v>129</v>
+        <v>167</v>
       </c>
       <c r="G38" s="26"/>
       <c r="H38" s="26"/>
@@ -2594,36 +3302,36 @@
         <v>53</v>
       </c>
       <c r="E41" s="27" t="s">
-        <v>130</v>
+        <v>168</v>
       </c>
       <c r="F41" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G41" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H41" s="15" t="s">
-        <v>131</v>
+        <v>169</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B42" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C42" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D42" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E42" s="25" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F42" s="26" t="s">
-        <v>132</v>
+        <v>170</v>
       </c>
       <c r="G42" s="26"/>
       <c r="H42" s="26"/>
@@ -2642,36 +3350,36 @@
         <v>46</v>
       </c>
       <c r="E44" s="22" t="s">
-        <v>119</v>
+        <v>157</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>120</v>
+        <v>158</v>
       </c>
       <c r="G44" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>133</v>
+        <v>171</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B45" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C45" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D45" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E45" s="25" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F45" s="26" t="s">
-        <v>134</v>
+        <v>172</v>
       </c>
       <c r="G45" s="26"/>
       <c r="H45" s="26"/>
@@ -2690,192 +3398,192 @@
         <v>16</v>
       </c>
       <c r="E47" s="27" t="s">
-        <v>88</v>
+        <v>126</v>
       </c>
       <c r="F47" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G47" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H47" s="15" t="s">
-        <v>90</v>
+        <v>128</v>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C48" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D48" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E48" s="27" t="s">
-        <v>135</v>
+        <v>173</v>
       </c>
       <c r="F48" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G48" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H48" s="15" t="s">
-        <v>136</v>
+        <v>174</v>
       </c>
     </row>
     <row r="49" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C49" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D49" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E49" s="27" t="s">
-        <v>137</v>
+        <v>175</v>
       </c>
       <c r="F49" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H49" s="15" t="s">
-        <v>138</v>
+        <v>176</v>
       </c>
     </row>
     <row r="50" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C50" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D50" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E50" s="27" t="s">
-        <v>110</v>
+        <v>148</v>
       </c>
       <c r="F50" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G50" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H50" s="15" t="s">
-        <v>139</v>
+        <v>177</v>
       </c>
     </row>
     <row r="51" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B51" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C51" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D51" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E51" s="27" t="s">
-        <v>140</v>
+        <v>178</v>
       </c>
       <c r="F51" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G51" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H51" s="15" t="s">
-        <v>141</v>
+        <v>179</v>
       </c>
     </row>
     <row r="52" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C52" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D52" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E52" s="27" t="s">
-        <v>142</v>
+        <v>180</v>
       </c>
       <c r="F52" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G52" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H52" s="15" t="s">
-        <v>143</v>
+        <v>181</v>
       </c>
     </row>
     <row r="53" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C53" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D53" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E53" s="27" t="s">
-        <v>92</v>
+        <v>130</v>
       </c>
       <c r="F53" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G53" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H53" s="15" t="s">
-        <v>144</v>
+        <v>182</v>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B54" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C54" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D54" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E54" s="25" t="s">
-        <v>117</v>
+        <v>155</v>
       </c>
       <c r="F54" s="26" t="s">
-        <v>145</v>
+        <v>183</v>
       </c>
       <c r="G54" s="26"/>
       <c r="H54" s="26"/>
@@ -2894,218 +3602,218 @@
         <v>42</v>
       </c>
       <c r="E56" s="22" t="s">
-        <v>119</v>
+        <v>157</v>
       </c>
       <c r="F56" s="8" t="s">
-        <v>120</v>
+        <v>158</v>
       </c>
       <c r="G56" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>146</v>
+        <v>184</v>
       </c>
     </row>
     <row r="57" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C57" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E57" s="22" t="s">
-        <v>88</v>
+        <v>126</v>
       </c>
       <c r="F57" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G57" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H57" s="9" t="s">
-        <v>147</v>
+        <v>185</v>
       </c>
     </row>
     <row r="58" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C58" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E58" s="22" t="s">
-        <v>135</v>
+        <v>173</v>
       </c>
       <c r="F58" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G58" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H58" s="9" t="s">
-        <v>148</v>
+        <v>186</v>
       </c>
     </row>
     <row r="59" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C59" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E59" s="22" t="s">
-        <v>137</v>
+        <v>175</v>
       </c>
       <c r="F59" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G59" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H59" s="9" t="s">
-        <v>149</v>
+        <v>187</v>
       </c>
     </row>
     <row r="60" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C60" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E60" s="22" t="s">
-        <v>110</v>
+        <v>148</v>
       </c>
       <c r="F60" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G60" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H60" s="9" t="s">
-        <v>124</v>
+        <v>162</v>
       </c>
     </row>
     <row r="61" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C61" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E61" s="22" t="s">
-        <v>140</v>
+        <v>178</v>
       </c>
       <c r="F61" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G61" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H61" s="9" t="s">
-        <v>150</v>
+        <v>188</v>
       </c>
     </row>
     <row r="62" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C62" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E62" s="22" t="s">
-        <v>142</v>
+        <v>180</v>
       </c>
       <c r="F62" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G62" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H62" s="9" t="s">
-        <v>151</v>
+        <v>189</v>
       </c>
     </row>
     <row r="63" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C63" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E63" s="22" t="s">
-        <v>92</v>
+        <v>130</v>
       </c>
       <c r="F63" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G63" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H63" s="9" t="s">
-        <v>152</v>
+        <v>190</v>
       </c>
     </row>
     <row r="64" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B64" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C64" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D64" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E64" s="25" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F64" s="26" t="s">
-        <v>153</v>
+        <v>191</v>
       </c>
       <c r="G64" s="26"/>
       <c r="H64" s="26"/>
@@ -3124,36 +3832,36 @@
         <v>46</v>
       </c>
       <c r="E66" s="27" t="s">
-        <v>119</v>
+        <v>157</v>
       </c>
       <c r="F66" s="14" t="s">
-        <v>120</v>
+        <v>158</v>
       </c>
       <c r="G66" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H66" s="15" t="s">
-        <v>133</v>
+        <v>171</v>
       </c>
     </row>
     <row r="67" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B67" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C67" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D67" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E67" s="25" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F67" s="26" t="s">
-        <v>154</v>
+        <v>192</v>
       </c>
       <c r="G67" s="26"/>
       <c r="H67" s="26"/>
@@ -3184,114 +3892,114 @@
         <v>53</v>
       </c>
       <c r="E70" s="22" t="s">
-        <v>142</v>
+        <v>180</v>
       </c>
       <c r="F70" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G70" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H70" s="9" t="s">
-        <v>155</v>
+        <v>193</v>
       </c>
     </row>
     <row r="71" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C71" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E71" s="22" t="s">
-        <v>156</v>
+        <v>194</v>
       </c>
       <c r="F71" s="8" t="s">
-        <v>120</v>
+        <v>158</v>
       </c>
       <c r="G71" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H71" s="9" t="s">
-        <v>157</v>
+        <v>195</v>
       </c>
     </row>
     <row r="72" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B72" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C72" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D72" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E72" s="22" t="s">
-        <v>130</v>
+        <v>168</v>
       </c>
       <c r="F72" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G72" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H72" s="9" t="s">
-        <v>158</v>
+        <v>196</v>
       </c>
     </row>
     <row r="73" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B73" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C73" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D73" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E73" s="22" t="s">
-        <v>115</v>
+        <v>153</v>
       </c>
       <c r="F73" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G73" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>159</v>
+        <v>197</v>
       </c>
     </row>
     <row r="74" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B74" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C74" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D74" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E74" s="25" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F74" s="26" t="s">
-        <v>160</v>
+        <v>198</v>
       </c>
       <c r="G74" s="26"/>
       <c r="H74" s="26"/>
@@ -3310,36 +4018,36 @@
         <v>46</v>
       </c>
       <c r="E76" s="27" t="s">
-        <v>119</v>
+        <v>157</v>
       </c>
       <c r="F76" s="14" t="s">
-        <v>120</v>
+        <v>158</v>
       </c>
       <c r="G76" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H76" s="15" t="s">
-        <v>161</v>
+        <v>199</v>
       </c>
     </row>
     <row r="77" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B77" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C77" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D77" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E77" s="25" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F77" s="26" t="s">
-        <v>162</v>
+        <v>200</v>
       </c>
       <c r="G77" s="26"/>
       <c r="H77" s="26"/>
@@ -3358,296 +4066,296 @@
         <v>16</v>
       </c>
       <c r="E79" s="22" t="s">
-        <v>156</v>
+        <v>194</v>
       </c>
       <c r="F79" s="8" t="s">
-        <v>120</v>
+        <v>158</v>
       </c>
       <c r="G79" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H79" s="9" t="s">
-        <v>163</v>
+        <v>201</v>
       </c>
     </row>
     <row r="80" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B80" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C80" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D80" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E80" s="22" t="s">
-        <v>164</v>
+        <v>202</v>
       </c>
       <c r="F80" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G80" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H80" s="9" t="s">
-        <v>165</v>
+        <v>203</v>
       </c>
     </row>
     <row r="81" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B81" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C81" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D81" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E81" s="22" t="s">
-        <v>166</v>
+        <v>204</v>
       </c>
       <c r="F81" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G81" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H81" s="9" t="s">
-        <v>167</v>
+        <v>205</v>
       </c>
     </row>
     <row r="82" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B82" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C82" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D82" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E82" s="22" t="s">
-        <v>168</v>
+        <v>206</v>
       </c>
       <c r="F82" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G82" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H82" s="9" t="s">
-        <v>169</v>
+        <v>207</v>
       </c>
     </row>
     <row r="83" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B83" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C83" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D83" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E83" s="22" t="s">
-        <v>170</v>
+        <v>208</v>
       </c>
       <c r="F83" s="8" t="s">
-        <v>171</v>
+        <v>209</v>
       </c>
       <c r="G83" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H83" s="9" t="s">
-        <v>172</v>
+        <v>210</v>
       </c>
     </row>
     <row r="84" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B84" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C84" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D84" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E84" s="22" t="s">
-        <v>173</v>
+        <v>211</v>
       </c>
       <c r="F84" s="8" t="s">
-        <v>171</v>
+        <v>209</v>
       </c>
       <c r="G84" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H84" s="9" t="s">
-        <v>174</v>
+        <v>212</v>
       </c>
     </row>
     <row r="85" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B85" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C85" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D85" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E85" s="22" t="s">
-        <v>175</v>
+        <v>213</v>
       </c>
       <c r="F85" s="8" t="s">
-        <v>120</v>
+        <v>158</v>
       </c>
       <c r="G85" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H85" s="9" t="s">
-        <v>176</v>
+        <v>214</v>
       </c>
     </row>
     <row r="86" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B86" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C86" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D86" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E86" s="22" t="s">
-        <v>177</v>
+        <v>215</v>
       </c>
       <c r="F86" s="8" t="s">
-        <v>171</v>
+        <v>209</v>
       </c>
       <c r="G86" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H86" s="9" t="s">
-        <v>178</v>
+        <v>216</v>
       </c>
     </row>
     <row r="87" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B87" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C87" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D87" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E87" s="22" t="s">
-        <v>179</v>
+        <v>217</v>
       </c>
       <c r="F87" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G87" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H87" s="9" t="s">
-        <v>180</v>
+        <v>218</v>
       </c>
     </row>
     <row r="88" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B88" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C88" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D88" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E88" s="22" t="s">
-        <v>181</v>
+        <v>219</v>
       </c>
       <c r="F88" s="8" t="s">
-        <v>182</v>
+        <v>220</v>
       </c>
       <c r="G88" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H88" s="9" t="s">
-        <v>183</v>
+        <v>221</v>
       </c>
     </row>
     <row r="89" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B89" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C89" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D89" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E89" s="22" t="s">
-        <v>115</v>
+        <v>153</v>
       </c>
       <c r="F89" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G89" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H89" s="9" t="s">
-        <v>116</v>
+        <v>154</v>
       </c>
     </row>
     <row r="90" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B90" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C90" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D90" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E90" s="25" t="s">
-        <v>117</v>
+        <v>155</v>
       </c>
       <c r="F90" s="26" t="s">
-        <v>184</v>
+        <v>222</v>
       </c>
       <c r="G90" s="26"/>
       <c r="H90" s="26"/>
@@ -3666,296 +4374,296 @@
         <v>42</v>
       </c>
       <c r="E92" s="27" t="s">
-        <v>119</v>
+        <v>157</v>
       </c>
       <c r="F92" s="14" t="s">
-        <v>120</v>
+        <v>158</v>
       </c>
       <c r="G92" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H92" s="15" t="s">
-        <v>185</v>
+        <v>223</v>
       </c>
     </row>
     <row r="93" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B93" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C93" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D93" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E93" s="27" t="s">
-        <v>164</v>
+        <v>202</v>
       </c>
       <c r="F93" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G93" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H93" s="15" t="s">
-        <v>165</v>
+        <v>203</v>
       </c>
     </row>
     <row r="94" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B94" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C94" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D94" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E94" s="27" t="s">
-        <v>166</v>
+        <v>204</v>
       </c>
       <c r="F94" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G94" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H94" s="15" t="s">
-        <v>186</v>
+        <v>224</v>
       </c>
     </row>
     <row r="95" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B95" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C95" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D95" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E95" s="27" t="s">
-        <v>168</v>
+        <v>206</v>
       </c>
       <c r="F95" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G95" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H95" s="15" t="s">
-        <v>187</v>
+        <v>225</v>
       </c>
     </row>
     <row r="96" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B96" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C96" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D96" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E96" s="27" t="s">
-        <v>170</v>
+        <v>208</v>
       </c>
       <c r="F96" s="14" t="s">
-        <v>171</v>
+        <v>209</v>
       </c>
       <c r="G96" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H96" s="15" t="s">
-        <v>172</v>
+        <v>210</v>
       </c>
     </row>
     <row r="97" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B97" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C97" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D97" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E97" s="27" t="s">
-        <v>173</v>
+        <v>211</v>
       </c>
       <c r="F97" s="14" t="s">
-        <v>171</v>
+        <v>209</v>
       </c>
       <c r="G97" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H97" s="15" t="s">
-        <v>188</v>
+        <v>226</v>
       </c>
     </row>
     <row r="98" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B98" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C98" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D98" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E98" s="27" t="s">
-        <v>175</v>
+        <v>213</v>
       </c>
       <c r="F98" s="14" t="s">
-        <v>120</v>
+        <v>158</v>
       </c>
       <c r="G98" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H98" s="15" t="s">
-        <v>189</v>
+        <v>227</v>
       </c>
     </row>
     <row r="99" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B99" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C99" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D99" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E99" s="27" t="s">
-        <v>177</v>
+        <v>215</v>
       </c>
       <c r="F99" s="14" t="s">
-        <v>171</v>
+        <v>209</v>
       </c>
       <c r="G99" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H99" s="15" t="s">
-        <v>190</v>
+        <v>228</v>
       </c>
     </row>
     <row r="100" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B100" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C100" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D100" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E100" s="27" t="s">
-        <v>179</v>
+        <v>217</v>
       </c>
       <c r="F100" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G100" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H100" s="15" t="s">
-        <v>191</v>
+        <v>229</v>
       </c>
     </row>
     <row r="101" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B101" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C101" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D101" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E101" s="27" t="s">
-        <v>181</v>
+        <v>219</v>
       </c>
       <c r="F101" s="14" t="s">
-        <v>182</v>
+        <v>220</v>
       </c>
       <c r="G101" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H101" s="15" t="s">
-        <v>192</v>
+        <v>230</v>
       </c>
     </row>
     <row r="102" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B102" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C102" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D102" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E102" s="27" t="s">
-        <v>115</v>
+        <v>153</v>
       </c>
       <c r="F102" s="14" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G102" s="30" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="H102" s="15" t="s">
-        <v>126</v>
+        <v>164</v>
       </c>
     </row>
     <row r="103" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B103" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C103" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D103" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E103" s="25" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F103" s="26" t="s">
-        <v>193</v>
+        <v>231</v>
       </c>
       <c r="G103" s="26"/>
       <c r="H103" s="26"/>
@@ -3974,62 +4682,62 @@
         <v>42</v>
       </c>
       <c r="E105" s="22" t="s">
-        <v>119</v>
+        <v>157</v>
       </c>
       <c r="F105" s="8" t="s">
-        <v>120</v>
+        <v>158</v>
       </c>
       <c r="G105" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H105" s="9" t="s">
-        <v>185</v>
+        <v>223</v>
       </c>
     </row>
     <row r="106" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B106" s="9" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C106" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D106" s="8" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E106" s="22" t="s">
-        <v>179</v>
+        <v>217</v>
       </c>
       <c r="F106" s="8" t="s">
-        <v>89</v>
+        <v>127</v>
       </c>
       <c r="G106" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H106" s="9" t="s">
-        <v>191</v>
+        <v>229</v>
       </c>
     </row>
     <row r="107" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B107" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C107" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D107" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E107" s="25" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F107" s="26" t="s">
-        <v>193</v>
+        <v>231</v>
       </c>
       <c r="G107" s="26"/>
       <c r="H107" s="26"/>
@@ -4048,62 +4756,62 @@
         <v>42</v>
       </c>
       <c r="E109" s="27" t="s">
-        <v>119</v>
+        <v>157</v>
       </c>
       <c r="F109" s="14" t="s">
-        <v>120</v>
+        <v>158</v>
       </c>
       <c r="G109" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H109" s="15" t="s">
-        <v>185</v>
+        <v>223</v>
       </c>
     </row>
     <row r="110" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" s="12" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B110" s="15" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C110" s="28" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D110" s="14" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="E110" s="27" t="s">
-        <v>181</v>
+        <v>219</v>
       </c>
       <c r="F110" s="14" t="s">
-        <v>182</v>
+        <v>220</v>
       </c>
       <c r="G110" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H110" s="15" t="s">
-        <v>194</v>
+        <v>232</v>
       </c>
     </row>
     <row r="111" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B111" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C111" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D111" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E111" s="25" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F111" s="26" t="s">
-        <v>195</v>
+        <v>233</v>
       </c>
       <c r="G111" s="26"/>
       <c r="H111" s="26"/>
@@ -4122,42 +4830,1500 @@
         <v>46</v>
       </c>
       <c r="E113" s="22" t="s">
-        <v>119</v>
+        <v>157</v>
       </c>
       <c r="F113" s="8" t="s">
-        <v>120</v>
+        <v>158</v>
       </c>
       <c r="G113" s="23" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H113" s="9" t="s">
-        <v>161</v>
+        <v>199</v>
       </c>
     </row>
     <row r="114" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B114" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C114" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="D114" s="25" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E114" s="25" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F114" s="26" t="s">
-        <v>196</v>
+        <v>234</v>
       </c>
       <c r="G114" s="26"/>
       <c r="H114" s="26"/>
     </row>
+    <row r="116" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A116" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B116" s="4"/>
+      <c r="C116" s="4"/>
+      <c r="D116" s="4"/>
+      <c r="E116" s="4"/>
+      <c r="F116" s="4"/>
+      <c r="G116" s="4"/>
+      <c r="H116" s="4"/>
+    </row>
+    <row r="117" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>129</v>
+      </c>
+      <c r="B117" t="s">
+        <v>129</v>
+      </c>
+      <c r="C117" t="s">
+        <v>129</v>
+      </c>
+      <c r="D117" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="E117" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="F117" s="26" t="s">
+        <v>235</v>
+      </c>
+      <c r="G117" s="26"/>
+      <c r="H117" s="26"/>
+    </row>
+    <row r="119" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A119" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B119" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="C119" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D119" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E119" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="F119" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="G119" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H119" s="9" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="120" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>129</v>
+      </c>
+      <c r="B120" t="s">
+        <v>129</v>
+      </c>
+      <c r="C120" t="s">
+        <v>129</v>
+      </c>
+      <c r="D120" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="E120" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="F120" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="G120" s="26"/>
+      <c r="H120" s="26"/>
+    </row>
+    <row r="122" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A122" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B122" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C122" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D122" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="E122" s="27" t="s">
+        <v>238</v>
+      </c>
+      <c r="F122" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="G122" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H122" s="15" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="123" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A123" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B123" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C123" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="D123" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="E123" s="27" t="s">
+        <v>204</v>
+      </c>
+      <c r="F123" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="G123" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H123" s="15" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="124" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A124" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B124" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C124" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="D124" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="E124" s="27" t="s">
+        <v>241</v>
+      </c>
+      <c r="F124" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="G124" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H124" s="15" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="125" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A125" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B125" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C125" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="D125" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="E125" s="27" t="s">
+        <v>243</v>
+      </c>
+      <c r="F125" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="G125" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H125" s="15" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="126" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A126" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B126" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C126" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="D126" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="E126" s="27" t="s">
+        <v>245</v>
+      </c>
+      <c r="F126" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="G126" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H126" s="15" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="127" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A127" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B127" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C127" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="D127" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="E127" s="27" t="s">
+        <v>247</v>
+      </c>
+      <c r="F127" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="G127" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H127" s="15" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="128" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>129</v>
+      </c>
+      <c r="B128" t="s">
+        <v>129</v>
+      </c>
+      <c r="C128" t="s">
+        <v>129</v>
+      </c>
+      <c r="D128" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="E128" s="25" t="s">
+        <v>155</v>
+      </c>
+      <c r="F128" s="26" t="s">
+        <v>249</v>
+      </c>
+      <c r="G128" s="26"/>
+      <c r="H128" s="26"/>
+    </row>
+    <row r="130" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A130" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B130" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="C130" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D130" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E130" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="F130" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="G130" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H130" s="9" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="131" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A131" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B131" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C131" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D131" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E131" s="22" t="s">
+        <v>238</v>
+      </c>
+      <c r="F131" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="G131" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H131" s="9" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="132" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A132" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B132" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C132" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D132" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E132" s="22" t="s">
+        <v>204</v>
+      </c>
+      <c r="F132" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="G132" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H132" s="9" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="133" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A133" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B133" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C133" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D133" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E133" s="22" t="s">
+        <v>241</v>
+      </c>
+      <c r="F133" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="G133" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H133" s="9" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="134" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A134" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B134" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C134" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D134" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E134" s="22" t="s">
+        <v>243</v>
+      </c>
+      <c r="F134" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="G134" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H134" s="9" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="135" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A135" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B135" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C135" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D135" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E135" s="22" t="s">
+        <v>245</v>
+      </c>
+      <c r="F135" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="G135" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H135" s="9" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="136" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A136" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B136" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C136" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D136" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E136" s="22" t="s">
+        <v>247</v>
+      </c>
+      <c r="F136" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="G136" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H136" s="9" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="137" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>129</v>
+      </c>
+      <c r="B137" t="s">
+        <v>129</v>
+      </c>
+      <c r="C137" t="s">
+        <v>129</v>
+      </c>
+      <c r="D137" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="E137" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="F137" s="26" t="s">
+        <v>250</v>
+      </c>
+      <c r="G137" s="26"/>
+      <c r="H137" s="26"/>
+    </row>
+    <row r="139" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A139" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B139" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="C139" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="D139" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="E139" s="27" t="s">
+        <v>157</v>
+      </c>
+      <c r="F139" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="G139" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H139" s="15" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="140" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>129</v>
+      </c>
+      <c r="B140" t="s">
+        <v>129</v>
+      </c>
+      <c r="C140" t="s">
+        <v>129</v>
+      </c>
+      <c r="D140" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="E140" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="F140" s="26" t="s">
+        <v>251</v>
+      </c>
+      <c r="G140" s="26"/>
+      <c r="H140" s="26"/>
+    </row>
+    <row r="142" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A142" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B142" s="4"/>
+      <c r="C142" s="4"/>
+      <c r="D142" s="4"/>
+      <c r="E142" s="4"/>
+      <c r="F142" s="4"/>
+      <c r="G142" s="4"/>
+      <c r="H142" s="4"/>
+    </row>
+    <row r="143" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>129</v>
+      </c>
+      <c r="B143" t="s">
+        <v>129</v>
+      </c>
+      <c r="C143" t="s">
+        <v>129</v>
+      </c>
+      <c r="D143" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="E143" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="F143" s="26" t="s">
+        <v>252</v>
+      </c>
+      <c r="G143" s="26"/>
+      <c r="H143" s="26"/>
+    </row>
+    <row r="145" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A145" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="B145" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="C145" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="D145" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="E145" s="27" t="s">
+        <v>157</v>
+      </c>
+      <c r="F145" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="G145" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H145" s="15" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="146" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>129</v>
+      </c>
+      <c r="B146" t="s">
+        <v>129</v>
+      </c>
+      <c r="C146" t="s">
+        <v>129</v>
+      </c>
+      <c r="D146" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="E146" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="F146" s="26" t="s">
+        <v>254</v>
+      </c>
+      <c r="G146" s="26"/>
+      <c r="H146" s="26"/>
+    </row>
+    <row r="148" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A148" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B148" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C148" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D148" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E148" s="22" t="s">
+        <v>255</v>
+      </c>
+      <c r="F148" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="G148" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H148" s="9" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="149" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A149" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B149" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C149" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D149" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E149" s="22" t="s">
+        <v>256</v>
+      </c>
+      <c r="F149" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="G149" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H149" s="9" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="150" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A150" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B150" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C150" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D150" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E150" s="22" t="s">
+        <v>257</v>
+      </c>
+      <c r="F150" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="G150" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H150" s="9" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="151" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A151" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B151" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C151" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D151" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E151" s="22" t="s">
+        <v>259</v>
+      </c>
+      <c r="F151" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="G151" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H151" s="9" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="152" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A152" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B152" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C152" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D152" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E152" s="22" t="s">
+        <v>261</v>
+      </c>
+      <c r="F152" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="G152" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H152" s="9" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="153" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A153" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B153" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C153" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D153" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E153" s="22" t="s">
+        <v>262</v>
+      </c>
+      <c r="F153" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="G153" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H153" s="9" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="154" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A154" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B154" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C154" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D154" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E154" s="22" t="s">
+        <v>264</v>
+      </c>
+      <c r="F154" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="G154" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H154" s="9" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="155" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>129</v>
+      </c>
+      <c r="B155" t="s">
+        <v>129</v>
+      </c>
+      <c r="C155" t="s">
+        <v>129</v>
+      </c>
+      <c r="D155" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="E155" s="25" t="s">
+        <v>155</v>
+      </c>
+      <c r="F155" s="26" t="s">
+        <v>265</v>
+      </c>
+      <c r="G155" s="26"/>
+      <c r="H155" s="26"/>
+    </row>
+    <row r="157" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A157" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="B157" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="C157" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="D157" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E157" s="27" t="s">
+        <v>157</v>
+      </c>
+      <c r="F157" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="G157" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H157" s="15" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="158" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A158" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B158" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C158" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="D158" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="E158" s="27" t="s">
+        <v>255</v>
+      </c>
+      <c r="F158" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="G158" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H158" s="15" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="159" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A159" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B159" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C159" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="D159" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="E159" s="27" t="s">
+        <v>256</v>
+      </c>
+      <c r="F159" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="G159" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H159" s="15" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="160" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A160" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B160" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C160" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="D160" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="E160" s="27" t="s">
+        <v>257</v>
+      </c>
+      <c r="F160" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="G160" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H160" s="15" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="161" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A161" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B161" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C161" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="D161" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="E161" s="27" t="s">
+        <v>259</v>
+      </c>
+      <c r="F161" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="G161" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H161" s="15" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="162" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A162" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B162" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C162" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="D162" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="E162" s="27" t="s">
+        <v>261</v>
+      </c>
+      <c r="F162" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="G162" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H162" s="15" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="163" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A163" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B163" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C163" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="D163" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="E163" s="27" t="s">
+        <v>262</v>
+      </c>
+      <c r="F163" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="G163" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H163" s="15" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="164" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A164" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B164" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C164" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="D164" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="E164" s="27" t="s">
+        <v>264</v>
+      </c>
+      <c r="F164" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="G164" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H164" s="15" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="165" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>129</v>
+      </c>
+      <c r="B165" t="s">
+        <v>129</v>
+      </c>
+      <c r="C165" t="s">
+        <v>129</v>
+      </c>
+      <c r="D165" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="E165" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="F165" s="26" t="s">
+        <v>266</v>
+      </c>
+      <c r="G165" s="26"/>
+      <c r="H165" s="26"/>
+    </row>
+    <row r="167" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A167" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B167" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="C167" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="D167" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E167" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="F167" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="G167" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H167" s="9" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="168" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>129</v>
+      </c>
+      <c r="B168" t="s">
+        <v>129</v>
+      </c>
+      <c r="C168" t="s">
+        <v>129</v>
+      </c>
+      <c r="D168" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="E168" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="F168" s="26" t="s">
+        <v>267</v>
+      </c>
+      <c r="G168" s="26"/>
+      <c r="H168" s="26"/>
+    </row>
+    <row r="170" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A170" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B170" s="4"/>
+      <c r="C170" s="4"/>
+      <c r="D170" s="4"/>
+      <c r="E170" s="4"/>
+      <c r="F170" s="4"/>
+      <c r="G170" s="4"/>
+      <c r="H170" s="4"/>
+    </row>
+    <row r="171" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>129</v>
+      </c>
+      <c r="B171" t="s">
+        <v>129</v>
+      </c>
+      <c r="C171" t="s">
+        <v>129</v>
+      </c>
+      <c r="D171" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="E171" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="F171" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G171" s="26"/>
+      <c r="H171" s="26"/>
+    </row>
+    <row r="173" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A173" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B173" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C173" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D173" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E173" s="22" t="s">
+        <v>269</v>
+      </c>
+      <c r="F173" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="G173" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H173" s="9" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="174" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A174" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B174" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C174" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D174" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E174" s="22" t="s">
+        <v>271</v>
+      </c>
+      <c r="F174" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="G174" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H174" s="9" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="175" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A175" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B175" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C175" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D175" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E175" s="22" t="s">
+        <v>273</v>
+      </c>
+      <c r="F175" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="G175" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H175" s="9" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="176" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A176" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B176" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C176" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D176" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E176" s="22" t="s">
+        <v>275</v>
+      </c>
+      <c r="F176" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="G176" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H176" s="9" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="177" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A177" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B177" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C177" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D177" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E177" s="22" t="s">
+        <v>277</v>
+      </c>
+      <c r="F177" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="G177" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="H177" s="9" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="178" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>129</v>
+      </c>
+      <c r="B178" t="s">
+        <v>129</v>
+      </c>
+      <c r="C178" t="s">
+        <v>129</v>
+      </c>
+      <c r="D178" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="E178" s="25" t="s">
+        <v>155</v>
+      </c>
+      <c r="F178" s="26" t="s">
+        <v>279</v>
+      </c>
+      <c r="G178" s="26"/>
+      <c r="H178" s="26"/>
+    </row>
+    <row r="180" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A180" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="B180" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C180" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="D180" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="E180" s="27" t="s">
+        <v>280</v>
+      </c>
+      <c r="F180" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="G180" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H180" s="15" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="181" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A181" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B181" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C181" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="D181" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="E181" s="27" t="s">
+        <v>282</v>
+      </c>
+      <c r="F181" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="G181" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H181" s="15" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="182" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>129</v>
+      </c>
+      <c r="B182" t="s">
+        <v>129</v>
+      </c>
+      <c r="C182" t="s">
+        <v>129</v>
+      </c>
+      <c r="D182" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="E182" s="25" t="s">
+        <v>155</v>
+      </c>
+      <c r="F182" s="26" t="s">
+        <v>285</v>
+      </c>
+      <c r="G182" s="26"/>
+      <c r="H182" s="26"/>
+    </row>
+    <row r="184" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A184" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B184" s="33" t="s">
+        <v>74</v>
+      </c>
+      <c r="C184" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D184" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E184" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="F184" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="G184" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H184" s="9" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="185" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A185" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B185" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C185" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D185" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E185" s="22" t="s">
+        <v>180</v>
+      </c>
+      <c r="F185" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="G185" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H185" s="9" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="186" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>129</v>
+      </c>
+      <c r="B186" t="s">
+        <v>129</v>
+      </c>
+      <c r="C186" t="s">
+        <v>129</v>
+      </c>
+      <c r="D186" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="E186" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="F186" s="26" t="s">
+        <v>288</v>
+      </c>
+      <c r="G186" s="26"/>
+      <c r="H186" s="26"/>
+    </row>
+    <row r="188" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A188" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="B188" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="C188" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="D188" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="E188" s="27" t="s">
+        <v>157</v>
+      </c>
+      <c r="F188" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="G188" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H188" s="15" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="189" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>129</v>
+      </c>
+      <c r="B189" t="s">
+        <v>129</v>
+      </c>
+      <c r="C189" t="s">
+        <v>129</v>
+      </c>
+      <c r="D189" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="E189" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="F189" s="26" t="s">
+        <v>289</v>
+      </c>
+      <c r="G189" s="26"/>
+      <c r="H189" s="26"/>
+    </row>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="43">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A5:H5"/>
@@ -4183,6 +6349,24 @@
     <mergeCell ref="F107:H107"/>
     <mergeCell ref="F111:H111"/>
     <mergeCell ref="F114:H114"/>
+    <mergeCell ref="A116:H116"/>
+    <mergeCell ref="F117:H117"/>
+    <mergeCell ref="F120:H120"/>
+    <mergeCell ref="F128:H128"/>
+    <mergeCell ref="F137:H137"/>
+    <mergeCell ref="F140:H140"/>
+    <mergeCell ref="A142:H142"/>
+    <mergeCell ref="F143:H143"/>
+    <mergeCell ref="F146:H146"/>
+    <mergeCell ref="F155:H155"/>
+    <mergeCell ref="F165:H165"/>
+    <mergeCell ref="F168:H168"/>
+    <mergeCell ref="A170:H170"/>
+    <mergeCell ref="F171:H171"/>
+    <mergeCell ref="F178:H178"/>
+    <mergeCell ref="F182:H182"/>
+    <mergeCell ref="F186:H186"/>
+    <mergeCell ref="F189:H189"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>